<commit_message>
Expand samples for every subject and verify safe repeat imports
</commit_message>
<xml_diff>
--- a/templates/hacknfix-cyber-questions-template.xlsx
+++ b/templates/hacknfix-cyber-questions-template.xlsx
@@ -1638,90 +1638,90 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="92" customHeight="1">
+    <row r="2" ht="108" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which action protects your account?</t>
+          <t xml:space="preserve">What should you do with recovery codes for an account?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">কোন কাজটি আপনার অ্যাকাউন্ট সুরক্ষিত রাখে?</t>
+          <t xml:space="preserve">অ্যাকাউন্টের রিকভারি কোড কীভাবে রাখবেন?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Share your password</t>
+          <t xml:space="preserve">Keep them in a secure place separate from the login device</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">পাসওয়ার্ড শেয়ার করা</t>
+          <t xml:space="preserve">লগইন ডিভাইস থেকে আলাদা নিরাপদ স্থানে রাখুন</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable two-factor authentication</t>
+          <t xml:space="preserve">Post them on social media</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">দুই ধাপের যাচাইকরণ চালু করা</t>
+          <t xml:space="preserve">সামাজিক মাধ্যমে প্রকাশ করুন</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Share them in a class group</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ক্লাসের গ্রুপে পাঠান</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A second verification step helps protect your account.</t>
+          <t xml:space="preserve">Recovery codes can unlock an account; keep them private and accessible to you.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">দ্বিতীয় যাচাইকরণ ধাপ অ্যাকাউন্ট সুরক্ষিত রাখতে সাহায্য করে।</t>
+          <t xml:space="preserve">রিকভারি কোড দিয়ে অ্যাকাউন্টে প্রবেশ করা যায়; গোপনে ও নিজের নাগালে রাখুন।</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">

</xml_diff>